<commit_message>
chore: add bfmaster matchup
</commit_message>
<xml_diff>
--- a/data/output/bayou.xlsx
+++ b/data/output/bayou.xlsx
@@ -36,31 +36,31 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Sealeo (Shadow) PS+S/BS 5/15/12</t>
+          <t>Blastoise RO+HC/SkB 4/8/15</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ice/water</t>
+          <t>water/none</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Lokix SkP+XS/TBl 4/15/13</t>
+          <t>Doublade SC+SSw/GB 6/15/15</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>bug/dark</t>
+          <t>steel/ghost</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Amoonguss A+GK/FoP 4/15/9</t>
+          <t>Amoonguss A+FoP/GK 4/15/9</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -72,7 +72,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Blastoise RO+HC/SkB 4/8/15</t>
+          <t>Seaking Pk+DR/IW 4/13/14</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -84,24 +84,24 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Seaking Pk+DR/IW 4/13/14</t>
+          <t>Skuntank (Shadow) PJ+Cr/TBl 4/15/14</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>water/none</t>
+          <t>poison/dark</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Skuntank PJ+Cr/TBl 4/15/14</t>
+          <t>Galvantula VS+D/Lu 4/15/9</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>poison/dark</t>
+          <t>bug/electric</t>
         </is>
       </c>
     </row>
@@ -141,7 +141,7 @@
         </is>
       </c>
       <c r="B3">
-        <v>189.77278173479093</v>
+        <v>173.72103521468983</v>
       </c>
     </row>
     <row r="4">
@@ -151,7 +151,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>125.90954773869346</v>
+        <v>109.53233830845771</v>
       </c>
     </row>
     <row r="5">
@@ -161,7 +161,7 @@
         </is>
       </c>
       <c r="B5">
-        <v>183.4717541291859</v>
+        <v>175.44283267343997</v>
       </c>
     </row>
     <row r="6">
@@ -171,7 +171,7 @@
         </is>
       </c>
       <c r="B6">
-        <v>761.047619047619</v>
+        <v>797.3541666666666</v>
       </c>
     </row>
     <row r="7">
@@ -181,7 +181,7 @@
         </is>
       </c>
       <c r="B7">
-        <v>16</v>
+        <v>82</v>
       </c>
     </row>
     <row r="8">
@@ -191,7 +191,7 @@
         </is>
       </c>
       <c r="B8">
-        <v>0.7619047619047619</v>
+        <v>0.8541666666666666</v>
       </c>
     </row>
     <row r="9">
@@ -201,7 +201,7 @@
         </is>
       </c>
       <c r="B9">
-        <v>7</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10">
@@ -211,7 +211,7 @@
         </is>
       </c>
       <c r="B10">
-        <v>703.9047619047619</v>
+        <v>733.2916666666666</v>
       </c>
     </row>
     <row r="11">
@@ -261,7 +261,7 @@
         </is>
       </c>
       <c r="B15">
-        <v>21</v>
+        <v>96</v>
       </c>
     </row>
     <row r="16">
@@ -271,7 +271,7 @@
         </is>
       </c>
       <c r="B16">
-        <v>19</v>
+        <v>94</v>
       </c>
     </row>
     <row r="17">
@@ -281,7 +281,7 @@
         </is>
       </c>
       <c r="B17">
-        <v>16</v>
+        <v>69</v>
       </c>
     </row>
     <row r="18">
@@ -331,7 +331,7 @@
         </is>
       </c>
       <c r="B22">
-        <v>86.02857142857144</v>
+        <v>86.7875</v>
       </c>
     </row>
     <row r="23">
@@ -341,7 +341,7 @@
         </is>
       </c>
       <c r="B23">
-        <v>74.8</v>
+        <v>73.2</v>
       </c>
     </row>
     <row r="24">
@@ -363,7 +363,7 @@
         </is>
       </c>
       <c r="B25">
-        <v>87.89999999999999</v>
+        <v>87.8</v>
       </c>
     </row>
     <row r="26">
@@ -383,7 +383,7 @@
         </is>
       </c>
       <c r="B27">
-        <v>0.09523809523809523</v>
+        <v>0.020833333333333332</v>
       </c>
     </row>
     <row r="28">
@@ -393,7 +393,7 @@
         </is>
       </c>
       <c r="B28">
-        <v>21</v>
+        <v>96</v>
       </c>
     </row>
     <row r="29">
@@ -403,7 +403,7 @@
         </is>
       </c>
       <c r="B29">
-        <v>654.9166666666666</v>
+        <v>661.0</v>
       </c>
     </row>
   </sheetData>
@@ -445,7 +445,7 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>7</v>
+        <v>32</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -462,7 +462,7 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>7</v>
+        <v>32</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -479,7 +479,7 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>7</v>
+        <v>32</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -531,22 +531,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>ABC</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>Galvantula VS+D/Lu 4/15/9</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Doublade SC+SSw/GB 6/15/15</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>Seaking Pk+DR/IW 4/13/14</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Blastoise RO+HC/SkB 4/8/15</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Lokix SkP+XS/TBl 4/15/13</t>
         </is>
       </c>
     </row>
@@ -556,22 +556,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ABC</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Sealeo (Shadow) PS+S/BS 5/15/12</t>
+          <t>Galvantula VS+D/Lu 4/15/9</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Amoonguss A+GK/FoP 4/15/9</t>
+          <t>Doublade SC+SSw/GB 6/15/15</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Lokix SkP+XS/TBl 4/15/13</t>
+          <t>Skuntank (Shadow) PJ+Cr/TBl 4/15/14</t>
         </is>
       </c>
     </row>
@@ -581,22 +581,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ABC</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Sealeo (Shadow) PS+S/BS 5/15/12</t>
+          <t>Blastoise RO+HC/SkB 4/8/15</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Seaking Pk+DR/IW 4/13/14</t>
+          <t>Doublade SC+SSw/GB 6/15/15</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Amoonguss A+GK/FoP 4/15/9</t>
+          <t>Skuntank (Shadow) PJ+Cr/TBl 4/15/14</t>
         </is>
       </c>
     </row>
@@ -606,17 +606,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ABC</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Skuntank PJ+Cr/TBl 4/15/14</t>
+          <t>Galvantula VS+D/Lu 4/15/9</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Seaking Pk+DR/IW 4/13/14</t>
+          <t>Doublade SC+SSw/GB 6/15/15</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -631,7 +631,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ABC</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -641,12 +641,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Blastoise RO+HC/SkB 4/8/15</t>
+          <t>Doublade SC+SSw/GB 6/15/15</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Amoonguss A+GK/FoP 4/15/9</t>
+          <t>Skuntank (Shadow) PJ+Cr/TBl 4/15/14</t>
         </is>
       </c>
     </row>
@@ -656,22 +656,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ABC</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
+          <t>Galvantula VS+D/Lu 4/15/9</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
           <t>Blastoise RO+HC/SkB 4/8/15</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Amoonguss A+GK/FoP 4/15/9</t>
-        </is>
-      </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Lokix SkP+XS/TBl 4/15/13</t>
+          <t>Skuntank (Shadow) PJ+Cr/TBl 4/15/14</t>
         </is>
       </c>
     </row>
@@ -681,22 +681,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ABC</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Skuntank PJ+Cr/TBl 4/15/14</t>
+          <t>Galvantula VS+D/Lu 4/15/9</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Sealeo (Shadow) PS+S/BS 5/15/12</t>
+          <t>Seaking Pk+DR/IW 4/13/14</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Amoonguss A+GK/FoP 4/15/9</t>
+          <t>Blastoise RO+HC/SkB 4/8/15</t>
         </is>
       </c>
     </row>
@@ -706,22 +706,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ABC</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Skuntank PJ+Cr/TBl 4/15/14</t>
+          <t>Seaking Pk+DR/IW 4/13/14</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Seaking Pk+DR/IW 4/13/14</t>
+          <t>Doublade SC+SSw/GB 6/15/15</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Amoonguss A+GK/FoP 4/15/9</t>
+          <t>Blastoise RO+HC/SkB 4/8/15</t>
         </is>
       </c>
     </row>
@@ -731,7 +731,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ABC</t>
+          <t>ABB</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -741,12 +741,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Amoonguss A+GK/FoP 4/15/9</t>
+          <t>Doublade SC+SSw/GB 6/15/15</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Lokix SkP+XS/TBl 4/15/13</t>
+          <t>Amoonguss A+FoP/GK 4/15/9</t>
         </is>
       </c>
     </row>
@@ -756,22 +756,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ABC</t>
+          <t>ABA</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Skuntank PJ+Cr/TBl 4/15/14</t>
+          <t>Galvantula VS+D/Lu 4/15/9</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Blastoise RO+HC/SkB 4/8/15</t>
+          <t>Seaking Pk+DR/IW 4/13/14</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Amoonguss A+GK/FoP 4/15/9</t>
+          <t>Amoonguss A+FoP/GK 4/15/9</t>
         </is>
       </c>
     </row>
@@ -807,7 +807,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Blastoise RO+HC/SkB 4/8/15</t>
+          <t>Pelipper WA+WBW/Hu 6/15/14</t>
         </is>
       </c>
       <c r="B2">
@@ -818,7 +818,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2-shield only Amoonguss A+GK/FoP 4/15/9</t>
+          <t>1-shield only Galvantula VS+D/Lu 4/15/9</t>
         </is>
       </c>
     </row>

</xml_diff>